<commit_message>
Improve survey data upload and processing with new file format support
Refactor the data upload and processing pipeline to support .docx files, unify file handling into a single upload interface, and enhance the quality reporting mechanism.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 1f7e2626-b96d-4407-a3c6-c3ff9161cc2b
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: dd982d60-4976-4f83-9a4b-fda7fb111472
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/bfe30bdd-353b-4a34-a48b-6024fd0147dc/1f7e2626-b96d-4407-a3c6-c3ff9161cc2b/euxdBiI
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/survey-insight-engine/tests/fixtures/missing_sheet1.xlsx
+++ b/artifacts/survey-insight-engine/tests/fixtures/missing_sheet1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="IndexOnly" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IndexOnly" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>